<commit_message>
Docs: SC-5b review complete (28/28), OpenAlex adopted (Q14), epistemic prisms noted
- Decision table: all 28 KEEP/RELINK lines decided; new parents Vision Science,
  Condensed Matter Physics; Pharmacology Root; OpenAlex alignment columns.
- SC-5c design note §9-§11: OpenAlex = reference for roots and mid-level domains
  (skos:closeMatch in SC-5b); colour models as DomainModel providers; Fourier
  Transform; future work: epistemological prisms.
No ontology change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015d5XtJTHoDrSjoqCKadpMN
</commit_message>
<xml_diff>
--- a/ontology/docs/_01_Worksite/WS-5/SC-5b/SC-5b_Subdomains_Decision_Table.xlsx
+++ b/ontology/docs/_01_Worksite/WS-5/SC-5b/SC-5b_Subdomains_Decision_Table.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1054" uniqueCount="533">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1082" uniqueCount="556">
   <si>
     <t xml:space="preserve">SC-5b — m1:subdomains strings on domain classes → decision per line</t>
   </si>
@@ -507,7 +507,7 @@
     <t xml:space="preserve">Signal Engineering</t>
   </si>
   <si>
-    <t xml:space="preserve">ext:electronics:SignalProcessing</t>
+    <t xml:space="preserve">dom:SignalProcessing</t>
   </si>
   <si>
     <t xml:space="preserve">Metrology</t>
@@ -532,16 +532,20 @@
 ext:electronics:Electronics</t>
   </si>
   <si>
-    <t xml:space="preserve">ext:electronics:Electronics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Two parents; Mathematics dangling</t>
+    <t xml:space="preserve">ext:electronics:Electronics
+dom:ComputerScience</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DECIDED Michel 2026-10-14: ⊑ Electronics (analog) + Computer Science (digital); closeMatch OpenAlex 1711; requires Fourier Transform (a DomainContract provider, belongsToDomain Mathematics)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">⊑ Electronics + Computer Science; requires Fourier Transform</t>
   </si>
   <si>
     <t xml:space="preserve">TVTestPattern, Transistor</t>
   </si>
   <si>
-    <t xml:space="preserve">Mathematics</t>
+    <t xml:space="preserve">Fourier Transform (DomainMethod or DomainModel, belongsToDomain Mathematics), Mathematics</t>
   </si>
   <si>
     <t xml:space="preserve">subfield 1711 Signal Processing</t>
@@ -705,6 +709,9 @@
     <t xml:space="preserve">Listed under Philosophy and Mythology; Mythology primary</t>
   </si>
   <si>
+    <t xml:space="preserve">OK (⊑ Mythology)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Descriptive, Explanatory</t>
   </si>
   <si>
@@ -747,6 +754,9 @@
     <t xml:space="preserve">ButterflyMetamorphosis; an M0 already cites m1.ext:biology:DevelopmentalBiology</t>
   </si>
   <si>
+    <t xml:space="preserve">OK (⊑ Biology)</t>
+  </si>
+  <si>
     <t xml:space="preserve">ButterflyMetamorphosis</t>
   </si>
   <si>
@@ -793,6 +803,9 @@
   </si>
   <si>
     <t xml:space="preserve">⊑ Physiology rather than Biology directly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OK (⊑ Physiology ⊑ Biology) — deliberate divergence from OpenAlex (sibling)</t>
   </si>
   <si>
     <t xml:space="preserve">subfield 1310 Endocrinology (also 2712, 2807)</t>
@@ -972,9 +985,15 @@
     <t xml:space="preserve">Listed under Chemistry and Physics (+4 combos); Physics primary, Chemistry via Physical Chemistry</t>
   </si>
   <si>
+    <t xml:space="preserve">OK (⊑ Physics)</t>
+  </si>
+  <si>
     <t xml:space="preserve">FireTriangle, FourStrokeEngine</t>
   </si>
   <si>
+    <t xml:space="preserve">Mathematics</t>
+  </si>
+  <si>
     <t xml:space="preserve">— (topics only)</t>
   </si>
   <si>
@@ -1053,6 +1072,9 @@
     <t xml:space="preserve">ext:education:InstructionalDesign</t>
   </si>
   <si>
+    <t xml:space="preserve">OK (⊑ Education)</t>
+  </si>
+  <si>
     <t xml:space="preserve">TPACK</t>
   </si>
   <si>
@@ -1089,16 +1111,25 @@
     <t xml:space="preserve">Semiconductor Physics</t>
   </si>
   <si>
+    <t xml:space="preserve">ext:electronics:Electronics</t>
+  </si>
+  <si>
     <t xml:space="preserve">ext:physics:SemiconductorPhysics</t>
   </si>
   <si>
-    <t xml:space="preserve">Two parents; Transistor</t>
+    <t xml:space="preserve">ext:physics:CondensedMatterPhysics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DECIDED Michel 2026-10-14: ⊑ Condensed Matter Physics (OpenAlex 3104) ⊑ Physics; requires Quantum Mechanics. Electronic Components ⊑ Electronics requires Semiconductor Physics (SC-5c). Transistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">⊑ Condensed Matter Physics; requires Quantum Mechanics</t>
   </si>
   <si>
     <t xml:space="preserve">Transistor</t>
   </si>
   <si>
-    <t xml:space="preserve">Electronics (inverse: Electronics requires it?)</t>
+    <t xml:space="preserve">Quantum Mechanics; [Electronic Components ⊑ Electronics requires Semiconductor Physics]</t>
   </si>
   <si>
     <t xml:space="preserve">— (topic T10472 Semiconductor materials and devices)</t>
@@ -1114,6 +1145,9 @@
   </si>
   <si>
     <t xml:space="preserve">ext:electronics:AnalogElectronics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OK (⊑ Electronics)</t>
   </si>
   <si>
     <t xml:space="preserve">Semiconductor Physics, Circuit Theory</t>
@@ -1159,6 +1193,9 @@
     <t xml:space="preserve">Two parents</t>
   </si>
   <si>
+    <t xml:space="preserve">OK (⊑ Geology + Physics); Geology closeMatch OpenAlex field 19</t>
+  </si>
+  <si>
     <t xml:space="preserve">PlateTectonics</t>
   </si>
   <si>
@@ -1241,7 +1278,7 @@
     <t xml:space="preserve">ext:optics:Optics</t>
   </si>
   <si>
-    <t xml:space="preserve">ext:optics:ColorScience</t>
+    <t xml:space="preserve">dom:ColorScience</t>
   </si>
   <si>
     <t xml:space="preserve">ColorSynthesis</t>
@@ -1250,13 +1287,22 @@
     <t xml:space="preserve">Color Science</t>
   </si>
   <si>
+    <t xml:space="preserve">dom:VisionScience</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DECIDED Michel 2026-10-14: colour is a perception model, not a property of light (cones, dyschromatopsia) → ⊑ Vision Science (Map side), requires Optics, Physiology. Colour spaces / gamut (RGB, CMY, CMYK, HSL instances) = m1:DomainModel of Color Science</t>
+  </si>
+  <si>
+    <t xml:space="preserve">⊑ Vision Science; requires Optics, Physiology</t>
+  </si>
+  <si>
     <t xml:space="preserve">Descriptive, Predictive</t>
   </si>
   <si>
     <t xml:space="preserve">CMY_Subtractive, ColorSynthesis, HSL_Additive, RGB_Additive</t>
   </si>
   <si>
-    <t xml:space="preserve">Physiology (vision)</t>
+    <t xml:space="preserve">Optics, Physiology (cones) — colour models (RGB, CMY, CMYK, HSL, gamut) = DomainModel</t>
   </si>
   <si>
     <t xml:space="preserve">Photography</t>
@@ -1278,6 +1324,9 @@
     <t xml:space="preserve">ext:optics:ImageFormation</t>
   </si>
   <si>
+    <t xml:space="preserve">OK (⊑ Optics)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Computer Graphics</t>
   </si>
   <si>
@@ -1394,6 +1443,18 @@
     <t xml:space="preserve">DECIDED: Root (Michel)</t>
   </si>
   <si>
+    <t xml:space="preserve">Vision Science</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DECIDED (Michel 2026-10-14): parent of Color Science; closeMatch OpenAlex subfield 2809 Sensory Systems</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condensed Matter Physics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DECIDED (Michel 2026-10-14): parent of Semiconductor Physics; closeMatch OpenAlex subfield 3104</t>
+  </si>
+  <si>
     <t xml:space="preserve">Card Game</t>
   </si>
   <si>
@@ -1475,9 +1536,6 @@
     <t xml:space="preserve">ext:physics:OrderParameter</t>
   </si>
   <si>
-    <t xml:space="preserve">Condensed Matter Physics</t>
-  </si>
-  <si>
     <t xml:space="preserve">Quantum Field Theory</t>
   </si>
   <si>
@@ -1632,6 +1690,18 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-12 (Michel, final): three relations — subClassOf (n parents, is-a-kind-of), m1:requires (relies on), Hybrid via m1:hybridOf (identity IS the crossing, e.g. Biomimetics) used judiciously, only where subClassOf and requires do not fit. Scope = computed view Root/Branch/Hybrid. SC-5b creates subClassOf only; requires/hybridOf/facets in SC-5c. See SC-5c design note.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">External reference vocabulary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OpenAlex (v2, ASJC-based) as the alignment reference for roots and mid-level domains, skos:closeMatch to https://openalex.org/fields/&lt;id&gt; or /subfields/&lt;id&gt;; Wikidata and specialist thesauri for finer levels. Divergences kept only with a written reason (e.g. Endocrinology ⊑ Physiology).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-13: ADOPTED (Michel). OpenAlex = reference for roots and mid-level; skos:closeMatch added in SC-5b on the lines that have an OpenAlex field/subfield; Wikidata for finer levels and the divergence rule in SC-5c.</t>
   </si>
   <si>
     <t xml:space="preserve">Q8</t>
@@ -2195,7 +2265,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T150"/>
+  <dimension ref="A1:T152"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -3648,7 +3718,7 @@
       <c r="S39" s="4"/>
       <c r="T39" s="7"/>
     </row>
-    <row r="40" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="n">
         <v>35</v>
       </c>
@@ -3670,7 +3740,9 @@
       <c r="G40" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="H40" s="7"/>
+      <c r="H40" s="7" t="s">
+        <v>168</v>
+      </c>
       <c r="I40" s="7"/>
       <c r="J40" s="4" t="s">
         <v>57</v>
@@ -3681,22 +3753,22 @@
       </c>
       <c r="M40" s="7"/>
       <c r="N40" s="4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="O40" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="P40" s="4" t="s">
         <v>36</v>
       </c>
       <c r="Q40" s="4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="R40" s="4" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="S40" s="4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="T40" s="7"/>
     </row>
@@ -3705,10 +3777,10 @@
         <v>36</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D41" s="6" t="s">
         <v>25</v>
@@ -3716,7 +3788,7 @@
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H41" s="7"/>
       <c r="I41" s="7"/>
@@ -3725,7 +3797,7 @@
       <c r="L41" s="4"/>
       <c r="M41" s="7"/>
       <c r="N41" s="4" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="O41" s="4"/>
       <c r="P41" s="4"/>
@@ -3739,10 +3811,10 @@
         <v>37</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D42" s="6" t="s">
         <v>25</v>
@@ -3750,7 +3822,7 @@
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H42" s="7"/>
       <c r="I42" s="7"/>
@@ -3771,20 +3843,20 @@
         <v>38</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D43" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E43" s="4"/>
       <c r="F43" s="4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H43" s="7"/>
       <c r="I43" s="7"/>
@@ -3805,20 +3877,20 @@
         <v>39</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D44" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E44" s="4"/>
       <c r="F44" s="4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H44" s="7"/>
       <c r="I44" s="7"/>
@@ -3839,23 +3911,23 @@
         <v>40</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D45" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E45" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="F45" s="4" t="s">
         <v>186</v>
-      </c>
-      <c r="F45" s="4" t="s">
-        <v>185</v>
       </c>
       <c r="G45" s="4"/>
       <c r="H45" s="7" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I45" s="7"/>
       <c r="J45" s="4" t="s">
@@ -3863,24 +3935,24 @@
       </c>
       <c r="K45" s="7"/>
       <c r="L45" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="M45" s="7"/>
       <c r="N45" s="4" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="O45" s="4"/>
       <c r="P45" s="4" t="s">
         <v>36</v>
       </c>
       <c r="Q45" s="4" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="R45" s="4" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="S45" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="T45" s="7"/>
     </row>
@@ -3889,10 +3961,10 @@
         <v>41</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D46" s="6" t="s">
         <v>25</v>
@@ -3900,7 +3972,7 @@
       <c r="E46" s="4"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H46" s="7"/>
       <c r="I46" s="7"/>
@@ -3909,7 +3981,7 @@
       <c r="L46" s="4"/>
       <c r="M46" s="7"/>
       <c r="N46" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="O46" s="4"/>
       <c r="P46" s="4"/>
@@ -3923,10 +3995,10 @@
         <v>42</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D47" s="6" t="s">
         <v>25</v>
@@ -3934,7 +4006,7 @@
       <c r="E47" s="4"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="H47" s="7"/>
       <c r="I47" s="7"/>
@@ -3955,17 +4027,17 @@
         <v>43</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D48" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E48" s="4"/>
       <c r="F48" s="4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G48" s="4" t="s">
         <v>26</v>
@@ -3989,20 +4061,20 @@
         <v>44</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D49" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E49" s="4"/>
       <c r="F49" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H49" s="7"/>
       <c r="I49" s="7"/>
@@ -4023,17 +4095,17 @@
         <v>45</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D50" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E50" s="4"/>
       <c r="F50" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G50" s="4" t="s">
         <v>26</v>
@@ -4057,17 +4129,17 @@
         <v>46</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D51" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E51" s="4"/>
       <c r="F51" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G51" s="4" t="s">
         <v>26</v>
@@ -4091,17 +4163,17 @@
         <v>47</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D52" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E52" s="4"/>
       <c r="F52" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G52" s="4" t="s">
         <v>26</v>
@@ -4125,20 +4197,20 @@
         <v>48</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D53" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E53" s="4"/>
       <c r="F53" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G53" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H53" s="7"/>
       <c r="I53" s="7"/>
@@ -4159,17 +4231,17 @@
         <v>49</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D54" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E54" s="4"/>
       <c r="F54" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G54" s="4" t="s">
         <v>26</v>
@@ -4193,25 +4265,25 @@
         <v>50</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D55" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G55" s="4" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H55" s="7" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="I55" s="7"/>
       <c r="J55" s="4" t="s">
@@ -4223,22 +4295,22 @@
       </c>
       <c r="M55" s="7"/>
       <c r="N55" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="O55" s="4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="P55" s="4" t="s">
         <v>36</v>
       </c>
       <c r="Q55" s="4" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="R55" s="4" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="S55" s="4" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="T55" s="7"/>
     </row>
@@ -4247,48 +4319,50 @@
         <v>51</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D56" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="G56" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="H56" s="7"/>
+        <v>223</v>
+      </c>
+      <c r="H56" s="7" t="s">
+        <v>224</v>
+      </c>
       <c r="I56" s="7"/>
       <c r="J56" s="4" t="s">
         <v>32</v>
       </c>
       <c r="K56" s="7"/>
       <c r="L56" s="4" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="M56" s="7"/>
       <c r="N56" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="O56" s="4"/>
       <c r="P56" s="4" t="s">
         <v>36</v>
       </c>
       <c r="Q56" s="4" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="R56" s="4" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="S56" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="T56" s="7"/>
     </row>
@@ -4297,10 +4371,10 @@
         <v>52</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D57" s="6" t="s">
         <v>25</v>
@@ -4308,7 +4382,7 @@
       <c r="E57" s="4"/>
       <c r="F57" s="4"/>
       <c r="G57" s="4" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="H57" s="7"/>
       <c r="I57" s="7"/>
@@ -4317,7 +4391,7 @@
       <c r="L57" s="4"/>
       <c r="M57" s="7"/>
       <c r="N57" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="O57" s="4"/>
       <c r="P57" s="4"/>
@@ -4331,7 +4405,7 @@
         <v>53</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C58" s="4" t="s">
         <v>77</v>
@@ -4340,7 +4414,7 @@
         <v>64</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
@@ -4363,7 +4437,7 @@
         <v>54</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>77</v>
@@ -4372,7 +4446,7 @@
         <v>64</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="F59" s="4"/>
       <c r="G59" s="4"/>
@@ -4395,7 +4469,7 @@
         <v>55</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C60" s="4" t="s">
         <v>77</v>
@@ -4406,7 +4480,7 @@
       <c r="E60" s="4"/>
       <c r="F60" s="4"/>
       <c r="G60" s="4" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="H60" s="7"/>
       <c r="I60" s="7"/>
@@ -4427,48 +4501,50 @@
         <v>56</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D61" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="H61" s="7"/>
+        <v>238</v>
+      </c>
+      <c r="H61" s="7" t="s">
+        <v>239</v>
+      </c>
       <c r="I61" s="7"/>
       <c r="J61" s="4" t="s">
         <v>32</v>
       </c>
       <c r="K61" s="7"/>
       <c r="L61" s="4" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="M61" s="7"/>
       <c r="N61" s="4" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="O61" s="4"/>
       <c r="P61" s="4" t="s">
         <v>36</v>
       </c>
       <c r="Q61" s="4" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="R61" s="4" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="S61" s="4" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="T61" s="7"/>
     </row>
@@ -4477,46 +4553,48 @@
         <v>57</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D62" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="G62" s="4"/>
-      <c r="H62" s="7"/>
+      <c r="H62" s="7" t="s">
+        <v>239</v>
+      </c>
       <c r="I62" s="7"/>
       <c r="J62" s="4" t="s">
         <v>32</v>
       </c>
       <c r="K62" s="7"/>
       <c r="L62" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="M62" s="7"/>
       <c r="N62" s="4" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="O62" s="4"/>
       <c r="P62" s="4" t="s">
         <v>36</v>
       </c>
       <c r="Q62" s="4" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="R62" s="4" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="S62" s="4" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="T62" s="7"/>
     </row>
@@ -4525,22 +4603,24 @@
         <v>58</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D63" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="G63" s="4"/>
-      <c r="H63" s="7"/>
+      <c r="H63" s="7" t="s">
+        <v>239</v>
+      </c>
       <c r="I63" s="7"/>
       <c r="J63" s="4" t="s">
         <v>32</v>
@@ -4551,70 +4631,72 @@
       </c>
       <c r="M63" s="7"/>
       <c r="N63" s="4" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="O63" s="4"/>
       <c r="P63" s="4" t="s">
         <v>36</v>
       </c>
       <c r="Q63" s="4" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="R63" s="4" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="S63" s="4" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="T63" s="7"/>
     </row>
-    <row r="64" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="4" t="n">
         <v>59</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D64" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E64" s="4" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="G64" s="4" t="s">
-        <v>252</v>
-      </c>
-      <c r="H64" s="7"/>
+        <v>255</v>
+      </c>
+      <c r="H64" s="7" t="s">
+        <v>256</v>
+      </c>
       <c r="I64" s="7"/>
       <c r="J64" s="4" t="s">
         <v>32</v>
       </c>
       <c r="K64" s="7"/>
       <c r="L64" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="M64" s="7"/>
       <c r="N64" s="4" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="O64" s="4"/>
       <c r="P64" s="4" t="s">
         <v>36</v>
       </c>
       <c r="Q64" s="4" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="R64" s="4" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="S64" s="4" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="T64" s="7"/>
     </row>
@@ -4623,20 +4705,20 @@
         <v>60</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D65" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E65" s="4"/>
       <c r="F65" s="4" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="G65" s="4" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="H65" s="7"/>
       <c r="I65" s="7"/>
@@ -4657,20 +4739,20 @@
         <v>61</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D66" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E66" s="4"/>
       <c r="F66" s="4" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="G66" s="4" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="H66" s="7"/>
       <c r="I66" s="7"/>
@@ -4691,20 +4773,20 @@
         <v>62</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D67" s="9" t="s">
         <v>64</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="F67" s="4"/>
       <c r="G67" s="4" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="H67" s="7"/>
       <c r="I67" s="7"/>
@@ -4725,10 +4807,10 @@
         <v>63</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D68" s="6" t="s">
         <v>25</v>
@@ -4736,7 +4818,7 @@
       <c r="E68" s="4"/>
       <c r="F68" s="4"/>
       <c r="G68" s="4" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="H68" s="7"/>
       <c r="I68" s="7"/>
@@ -4757,20 +4839,20 @@
         <v>64</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D69" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E69" s="4"/>
       <c r="F69" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="G69" s="4" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="H69" s="7"/>
       <c r="I69" s="7"/>
@@ -4791,20 +4873,20 @@
         <v>65</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D70" s="9" t="s">
         <v>64</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F70" s="4"/>
       <c r="G70" s="4" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="H70" s="7"/>
       <c r="I70" s="7"/>
@@ -4825,25 +4907,25 @@
         <v>66</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D71" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="G71" s="4" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="H71" s="7" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="I71" s="7"/>
       <c r="J71" s="4" t="s">
@@ -4855,22 +4937,22 @@
       </c>
       <c r="M71" s="7"/>
       <c r="N71" s="4" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="O71" s="4" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="P71" s="4" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="Q71" s="4" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="R71" s="4" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="S71" s="4" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="T71" s="7"/>
     </row>
@@ -4879,20 +4961,20 @@
         <v>67</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="D72" s="9" t="s">
         <v>64</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="F72" s="4"/>
       <c r="G72" s="4" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="H72" s="7"/>
       <c r="I72" s="7"/>
@@ -4913,20 +4995,20 @@
         <v>68</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="D73" s="9" t="s">
         <v>64</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="F73" s="4"/>
       <c r="G73" s="4" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="H73" s="7"/>
       <c r="I73" s="7"/>
@@ -4947,17 +5029,17 @@
         <v>69</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="D74" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E74" s="4"/>
       <c r="F74" s="4" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="G74" s="4" t="s">
         <v>44</v>
@@ -4981,10 +5063,10 @@
         <v>70</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="D75" s="6" t="s">
         <v>25</v>
@@ -4992,7 +5074,7 @@
       <c r="E75" s="4"/>
       <c r="F75" s="4"/>
       <c r="G75" s="4" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="H75" s="7"/>
       <c r="I75" s="7"/>
@@ -5013,10 +5095,10 @@
         <v>71</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="D76" s="6" t="s">
         <v>25</v>
@@ -5024,7 +5106,7 @@
       <c r="E76" s="4"/>
       <c r="F76" s="4"/>
       <c r="G76" s="4" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="H76" s="7"/>
       <c r="I76" s="7"/>
@@ -5045,10 +5127,10 @@
         <v>72</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="D77" s="6" t="s">
         <v>25</v>
@@ -5056,7 +5138,7 @@
       <c r="E77" s="4"/>
       <c r="F77" s="4"/>
       <c r="G77" s="4" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="H77" s="7"/>
       <c r="I77" s="7"/>
@@ -5077,16 +5159,16 @@
         <v>73</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="D78" s="9" t="s">
         <v>64</v>
       </c>
       <c r="E78" s="4" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="F78" s="4"/>
       <c r="G78" s="4"/>
@@ -5109,20 +5191,20 @@
         <v>74</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="D79" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E79" s="4"/>
       <c r="F79" s="4" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="G79" s="4" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="H79" s="7"/>
       <c r="I79" s="7"/>
@@ -5143,17 +5225,17 @@
         <v>75</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="D80" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E80" s="4"/>
       <c r="F80" s="4" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G80" s="4" t="s">
         <v>44</v>
@@ -5177,19 +5259,19 @@
         <v>76</v>
       </c>
       <c r="B81" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="C81" s="4" t="s">
         <v>299</v>
       </c>
-      <c r="C81" s="4" t="s">
-        <v>295</v>
-      </c>
       <c r="D81" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E81" s="4" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="G81" s="4" t="s">
         <v>26</v>
@@ -5213,17 +5295,17 @@
         <v>77</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="D82" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E82" s="4"/>
       <c r="F82" s="4" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="G82" s="4" t="s">
         <v>26</v>
@@ -5247,10 +5329,10 @@
         <v>78</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="D83" s="6" t="s">
         <v>25</v>
@@ -5258,7 +5340,7 @@
       <c r="E83" s="4"/>
       <c r="F83" s="4"/>
       <c r="G83" s="4" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="H83" s="7"/>
       <c r="I83" s="7"/>
@@ -5279,20 +5361,20 @@
         <v>79</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="D84" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E84" s="4"/>
       <c r="F84" s="4" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="G84" s="4" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="H84" s="7"/>
       <c r="I84" s="7"/>
@@ -5313,17 +5395,17 @@
         <v>80</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="D85" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E85" s="4"/>
       <c r="F85" s="4" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="G85" s="4" t="s">
         <v>44</v>
@@ -5350,21 +5432,23 @@
         <v>35</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="D86" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E86" s="4" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="F86" s="4" t="s">
         <v>160</v>
       </c>
       <c r="G86" s="4" t="s">
-        <v>310</v>
-      </c>
-      <c r="H86" s="7"/>
+        <v>314</v>
+      </c>
+      <c r="H86" s="7" t="s">
+        <v>315</v>
+      </c>
       <c r="I86" s="7"/>
       <c r="J86" s="4" t="s">
         <v>32</v>
@@ -5375,22 +5459,22 @@
       </c>
       <c r="M86" s="7"/>
       <c r="N86" s="4" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="O86" s="4" t="s">
-        <v>169</v>
+        <v>317</v>
       </c>
       <c r="P86" s="4" t="s">
         <v>36</v>
       </c>
       <c r="Q86" s="4" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="R86" s="4" t="s">
         <v>124</v>
       </c>
       <c r="S86" s="4" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="T86" s="7"/>
     </row>
@@ -5399,17 +5483,17 @@
         <v>82</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="D87" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E87" s="4"/>
       <c r="F87" s="4" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="G87" s="4" t="s">
         <v>26</v>
@@ -5433,17 +5517,17 @@
         <v>83</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="D88" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E88" s="4"/>
       <c r="F88" s="4" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="G88" s="4" t="s">
         <v>26</v>
@@ -5467,17 +5551,17 @@
         <v>84</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="D89" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E89" s="4"/>
       <c r="F89" s="4" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="G89" s="4" t="s">
         <v>26</v>
@@ -5501,10 +5585,10 @@
         <v>85</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="D90" s="6" t="s">
         <v>25</v>
@@ -5512,7 +5596,7 @@
       <c r="E90" s="4"/>
       <c r="F90" s="4"/>
       <c r="G90" s="4" t="s">
-        <v>319</v>
+        <v>325</v>
       </c>
       <c r="H90" s="7"/>
       <c r="I90" s="7"/>
@@ -5521,7 +5605,7 @@
       <c r="L90" s="4"/>
       <c r="M90" s="7"/>
       <c r="N90" s="4" t="s">
-        <v>320</v>
+        <v>326</v>
       </c>
       <c r="O90" s="4"/>
       <c r="P90" s="4"/>
@@ -5535,10 +5619,10 @@
         <v>86</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>321</v>
+        <v>327</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="D91" s="6" t="s">
         <v>25</v>
@@ -5546,7 +5630,7 @@
       <c r="E91" s="4"/>
       <c r="F91" s="4"/>
       <c r="G91" s="4" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="H91" s="7"/>
       <c r="I91" s="7"/>
@@ -5555,7 +5639,7 @@
       <c r="L91" s="4"/>
       <c r="M91" s="7"/>
       <c r="N91" s="4" t="s">
-        <v>320</v>
+        <v>326</v>
       </c>
       <c r="O91" s="4"/>
       <c r="P91" s="4"/>
@@ -5569,20 +5653,20 @@
         <v>87</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="D92" s="9" t="s">
         <v>64</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="F92" s="4"/>
       <c r="G92" s="4" t="s">
-        <v>326</v>
+        <v>332</v>
       </c>
       <c r="H92" s="7"/>
       <c r="I92" s="7"/>
@@ -5603,16 +5687,16 @@
         <v>88</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="D93" s="9" t="s">
         <v>64</v>
       </c>
       <c r="E93" s="4" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="F93" s="4"/>
       <c r="G93" s="4"/>
@@ -5635,20 +5719,20 @@
         <v>89</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="D94" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E94" s="4"/>
       <c r="F94" s="4" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="G94" s="4" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="H94" s="7"/>
       <c r="I94" s="7"/>
@@ -5669,17 +5753,17 @@
         <v>90</v>
       </c>
       <c r="B95" s="5" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="D95" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E95" s="4"/>
       <c r="F95" s="4" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="G95" s="4" t="s">
         <v>26</v>
@@ -5703,10 +5787,10 @@
         <v>91</v>
       </c>
       <c r="B96" s="5" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="D96" s="6" t="s">
         <v>25</v>
@@ -5714,7 +5798,7 @@
       <c r="E96" s="4"/>
       <c r="F96" s="4"/>
       <c r="G96" s="4" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="H96" s="7"/>
       <c r="I96" s="7"/>
@@ -5735,10 +5819,10 @@
         <v>92</v>
       </c>
       <c r="B97" s="5" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="D97" s="6" t="s">
         <v>25</v>
@@ -5767,22 +5851,24 @@
         <v>93</v>
       </c>
       <c r="B98" s="5" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="D98" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E98" s="4" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="G98" s="4"/>
-      <c r="H98" s="7"/>
+      <c r="H98" s="7" t="s">
+        <v>344</v>
+      </c>
       <c r="I98" s="7"/>
       <c r="J98" s="4" t="s">
         <v>121</v>
@@ -5793,20 +5879,20 @@
       </c>
       <c r="M98" s="7"/>
       <c r="N98" s="4" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="O98" s="4"/>
       <c r="P98" s="4" t="s">
         <v>36</v>
       </c>
       <c r="Q98" s="4" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="R98" s="4" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="S98" s="4" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
       <c r="T98" s="7"/>
     </row>
@@ -5815,24 +5901,26 @@
         <v>94</v>
       </c>
       <c r="B99" s="5" t="s">
+        <v>349</v>
+      </c>
+      <c r="C99" s="4" t="s">
         <v>342</v>
-      </c>
-      <c r="C99" s="4" t="s">
-        <v>336</v>
       </c>
       <c r="D99" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E99" s="4" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="G99" s="4" t="s">
-        <v>338</v>
-      </c>
-      <c r="H99" s="7"/>
+        <v>345</v>
+      </c>
+      <c r="H99" s="7" t="s">
+        <v>344</v>
+      </c>
       <c r="I99" s="7"/>
       <c r="J99" s="4" t="s">
         <v>57</v>
@@ -5843,22 +5931,22 @@
       </c>
       <c r="M99" s="7"/>
       <c r="N99" s="4" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="O99" s="4" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="P99" s="4" t="s">
         <v>36</v>
       </c>
       <c r="Q99" s="4" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
       <c r="R99" s="4" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="S99" s="4" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
       <c r="T99" s="7"/>
     </row>
@@ -5867,10 +5955,10 @@
         <v>95</v>
       </c>
       <c r="B100" s="5" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="C100" s="4" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="D100" s="6" t="s">
         <v>25</v>
@@ -5878,7 +5966,7 @@
       <c r="E100" s="4"/>
       <c r="F100" s="4"/>
       <c r="G100" s="4" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="H100" s="7"/>
       <c r="I100" s="7"/>
@@ -5899,16 +5987,16 @@
         <v>96</v>
       </c>
       <c r="B101" s="5" t="s">
-        <v>348</v>
+        <v>355</v>
       </c>
       <c r="C101" s="4" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="D101" s="9" t="s">
         <v>64</v>
       </c>
       <c r="E101" s="4" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="F101" s="4"/>
       <c r="G101" s="4"/>
@@ -5926,29 +6014,31 @@
       <c r="S101" s="4"/>
       <c r="T101" s="7"/>
     </row>
-    <row r="102" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="4" t="n">
         <v>97</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>349</v>
+        <v>356</v>
       </c>
       <c r="C102" s="4" t="s">
-        <v>166</v>
+        <v>357</v>
       </c>
       <c r="D102" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E102" s="4" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="F102" s="4" t="s">
-        <v>160</v>
+        <v>359</v>
       </c>
       <c r="G102" s="4" t="s">
-        <v>351</v>
-      </c>
-      <c r="H102" s="7"/>
+        <v>360</v>
+      </c>
+      <c r="H102" s="7" t="s">
+        <v>361</v>
+      </c>
       <c r="I102" s="7"/>
       <c r="J102" s="4" t="s">
         <v>32</v>
@@ -5959,22 +6049,22 @@
       </c>
       <c r="M102" s="7"/>
       <c r="N102" s="4" t="s">
-        <v>352</v>
+        <v>362</v>
       </c>
       <c r="O102" s="4" t="s">
-        <v>353</v>
+        <v>363</v>
       </c>
       <c r="P102" s="4" t="s">
         <v>36</v>
       </c>
       <c r="Q102" s="4" t="s">
-        <v>354</v>
+        <v>364</v>
       </c>
       <c r="R102" s="4" t="s">
-        <v>355</v>
+        <v>365</v>
       </c>
       <c r="S102" s="4" t="s">
-        <v>356</v>
+        <v>366</v>
       </c>
       <c r="T102" s="7"/>
     </row>
@@ -5983,22 +6073,24 @@
         <v>98</v>
       </c>
       <c r="B103" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="C103" s="4" t="s">
         <v>357</v>
-      </c>
-      <c r="C103" s="4" t="s">
-        <v>166</v>
       </c>
       <c r="D103" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E103" s="4" t="s">
-        <v>358</v>
+        <v>368</v>
       </c>
       <c r="F103" s="4" t="s">
-        <v>166</v>
+        <v>357</v>
       </c>
       <c r="G103" s="4"/>
-      <c r="H103" s="7"/>
+      <c r="H103" s="7" t="s">
+        <v>369</v>
+      </c>
       <c r="I103" s="7"/>
       <c r="J103" s="4" t="s">
         <v>57</v>
@@ -6009,22 +6101,22 @@
       </c>
       <c r="M103" s="7"/>
       <c r="N103" s="4" t="s">
-        <v>352</v>
+        <v>362</v>
       </c>
       <c r="O103" s="4" t="s">
-        <v>359</v>
+        <v>370</v>
       </c>
       <c r="P103" s="4" t="s">
         <v>36</v>
       </c>
       <c r="Q103" s="4" t="s">
-        <v>360</v>
+        <v>371</v>
       </c>
       <c r="R103" s="4" t="s">
-        <v>361</v>
+        <v>372</v>
       </c>
       <c r="S103" s="4" t="s">
-        <v>362</v>
+        <v>373</v>
       </c>
       <c r="T103" s="7"/>
     </row>
@@ -6033,20 +6125,20 @@
         <v>99</v>
       </c>
       <c r="B104" s="5" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="C104" s="4" t="s">
-        <v>166</v>
+        <v>357</v>
       </c>
       <c r="D104" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E104" s="4"/>
       <c r="F104" s="4" t="s">
-        <v>166</v>
+        <v>357</v>
       </c>
       <c r="G104" s="4" t="s">
-        <v>364</v>
+        <v>375</v>
       </c>
       <c r="H104" s="7"/>
       <c r="I104" s="7"/>
@@ -6062,27 +6154,29 @@
       <c r="S104" s="4"/>
       <c r="T104" s="7"/>
     </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="4" t="n">
         <v>100</v>
       </c>
       <c r="B105" s="5" t="s">
-        <v>365</v>
+        <v>376</v>
       </c>
       <c r="C105" s="4" t="s">
-        <v>166</v>
+        <v>357</v>
       </c>
       <c r="D105" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E105" s="4" t="s">
-        <v>366</v>
+        <v>377</v>
       </c>
       <c r="F105" s="4" t="s">
-        <v>166</v>
+        <v>357</v>
       </c>
       <c r="G105" s="4"/>
-      <c r="H105" s="7"/>
+      <c r="H105" s="7" t="s">
+        <v>369</v>
+      </c>
       <c r="I105" s="7"/>
       <c r="J105" s="4" t="s">
         <v>32</v>
@@ -6093,46 +6187,48 @@
       </c>
       <c r="M105" s="7"/>
       <c r="N105" s="4" t="s">
-        <v>352</v>
+        <v>362</v>
       </c>
       <c r="O105" s="4"/>
       <c r="P105" s="4" t="s">
         <v>36</v>
       </c>
       <c r="Q105" s="4" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="R105" s="4" t="s">
-        <v>367</v>
+        <v>378</v>
       </c>
       <c r="S105" s="4" t="s">
-        <v>362</v>
+        <v>373</v>
       </c>
       <c r="T105" s="7"/>
     </row>
-    <row r="106" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="106" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="4" t="n">
         <v>101</v>
       </c>
       <c r="B106" s="5" t="s">
-        <v>368</v>
+        <v>379</v>
       </c>
       <c r="C106" s="4" t="s">
-        <v>369</v>
+        <v>380</v>
       </c>
       <c r="D106" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E106" s="4" t="s">
-        <v>370</v>
+        <v>381</v>
       </c>
       <c r="F106" s="4" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="G106" s="4" t="s">
-        <v>372</v>
-      </c>
-      <c r="H106" s="7"/>
+        <v>383</v>
+      </c>
+      <c r="H106" s="7" t="s">
+        <v>384</v>
+      </c>
       <c r="I106" s="7"/>
       <c r="J106" s="4" t="s">
         <v>32</v>
@@ -6143,20 +6239,20 @@
       </c>
       <c r="M106" s="7"/>
       <c r="N106" s="4" t="s">
-        <v>373</v>
+        <v>385</v>
       </c>
       <c r="O106" s="4"/>
       <c r="P106" s="4" t="s">
         <v>36</v>
       </c>
       <c r="Q106" s="4" t="s">
-        <v>374</v>
+        <v>386</v>
       </c>
       <c r="R106" s="4" t="s">
-        <v>375</v>
+        <v>387</v>
       </c>
       <c r="S106" s="4" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="T106" s="7"/>
     </row>
@@ -6165,20 +6261,20 @@
         <v>102</v>
       </c>
       <c r="B107" s="5" t="s">
-        <v>377</v>
+        <v>389</v>
       </c>
       <c r="C107" s="4" t="s">
-        <v>369</v>
+        <v>380</v>
       </c>
       <c r="D107" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E107" s="4"/>
       <c r="F107" s="4" t="s">
-        <v>369</v>
+        <v>380</v>
       </c>
       <c r="G107" s="4" t="s">
-        <v>378</v>
+        <v>390</v>
       </c>
       <c r="H107" s="7"/>
       <c r="I107" s="7"/>
@@ -6199,20 +6295,20 @@
         <v>103</v>
       </c>
       <c r="B108" s="5" t="s">
-        <v>379</v>
+        <v>391</v>
       </c>
       <c r="C108" s="4" t="s">
-        <v>369</v>
+        <v>380</v>
       </c>
       <c r="D108" s="9" t="s">
         <v>64</v>
       </c>
       <c r="E108" s="4" t="s">
-        <v>380</v>
+        <v>392</v>
       </c>
       <c r="F108" s="4"/>
       <c r="G108" s="4" t="s">
-        <v>381</v>
+        <v>393</v>
       </c>
       <c r="H108" s="7"/>
       <c r="I108" s="7"/>
@@ -6233,17 +6329,17 @@
         <v>104</v>
       </c>
       <c r="B109" s="5" t="s">
-        <v>382</v>
+        <v>394</v>
       </c>
       <c r="C109" s="4" t="s">
-        <v>369</v>
+        <v>380</v>
       </c>
       <c r="D109" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E109" s="4"/>
       <c r="F109" s="4" t="s">
-        <v>370</v>
+        <v>381</v>
       </c>
       <c r="G109" s="4" t="s">
         <v>26</v>
@@ -6267,17 +6363,17 @@
         <v>105</v>
       </c>
       <c r="B110" s="5" t="s">
-        <v>383</v>
+        <v>395</v>
       </c>
       <c r="C110" s="4" t="s">
-        <v>369</v>
+        <v>380</v>
       </c>
       <c r="D110" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E110" s="4"/>
       <c r="F110" s="4" t="s">
-        <v>369</v>
+        <v>380</v>
       </c>
       <c r="G110" s="4" t="s">
         <v>26</v>
@@ -6301,17 +6397,17 @@
         <v>106</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>384</v>
+        <v>396</v>
       </c>
       <c r="C111" s="4" t="s">
-        <v>369</v>
+        <v>380</v>
       </c>
       <c r="D111" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E111" s="4"/>
       <c r="F111" s="4" t="s">
-        <v>369</v>
+        <v>380</v>
       </c>
       <c r="G111" s="4" t="s">
         <v>26</v>
@@ -6335,20 +6431,20 @@
         <v>107</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>385</v>
+        <v>397</v>
       </c>
       <c r="C112" s="4" t="s">
-        <v>369</v>
+        <v>380</v>
       </c>
       <c r="D112" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E112" s="4"/>
       <c r="F112" s="4" t="s">
-        <v>386</v>
+        <v>398</v>
       </c>
       <c r="G112" s="4" t="s">
-        <v>387</v>
+        <v>399</v>
       </c>
       <c r="H112" s="7"/>
       <c r="I112" s="7"/>
@@ -6369,10 +6465,10 @@
         <v>108</v>
       </c>
       <c r="B113" s="5" t="s">
-        <v>388</v>
+        <v>400</v>
       </c>
       <c r="C113" s="4" t="s">
-        <v>369</v>
+        <v>380</v>
       </c>
       <c r="D113" s="6" t="s">
         <v>25</v>
@@ -6380,7 +6476,7 @@
       <c r="E113" s="4"/>
       <c r="F113" s="4"/>
       <c r="G113" s="4" t="s">
-        <v>389</v>
+        <v>401</v>
       </c>
       <c r="H113" s="7"/>
       <c r="I113" s="7"/>
@@ -6401,20 +6497,20 @@
         <v>109</v>
       </c>
       <c r="B114" s="5" t="s">
-        <v>390</v>
+        <v>402</v>
       </c>
       <c r="C114" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D114" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E114" s="4"/>
       <c r="F114" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="G114" s="4" t="s">
-        <v>391</v>
+        <v>403</v>
       </c>
       <c r="H114" s="7"/>
       <c r="I114" s="7"/>
@@ -6435,20 +6531,20 @@
         <v>110</v>
       </c>
       <c r="B115" s="5" t="s">
-        <v>392</v>
+        <v>404</v>
       </c>
       <c r="C115" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D115" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E115" s="4"/>
       <c r="F115" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="G115" s="4" t="s">
-        <v>393</v>
+        <v>405</v>
       </c>
       <c r="H115" s="7"/>
       <c r="I115" s="7"/>
@@ -6469,20 +6565,20 @@
         <v>111</v>
       </c>
       <c r="B116" s="5" t="s">
-        <v>394</v>
+        <v>406</v>
       </c>
       <c r="C116" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D116" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E116" s="4"/>
       <c r="F116" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="G116" s="4" t="s">
-        <v>395</v>
+        <v>407</v>
       </c>
       <c r="H116" s="7"/>
       <c r="I116" s="7"/>
@@ -6503,10 +6599,10 @@
         <v>112</v>
       </c>
       <c r="B117" s="5" t="s">
-        <v>396</v>
+        <v>408</v>
       </c>
       <c r="C117" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D117" s="6" t="s">
         <v>25</v>
@@ -6514,7 +6610,7 @@
       <c r="E117" s="4"/>
       <c r="F117" s="4"/>
       <c r="G117" s="4" t="s">
-        <v>397</v>
+        <v>409</v>
       </c>
       <c r="H117" s="7"/>
       <c r="I117" s="7"/>
@@ -6535,16 +6631,16 @@
         <v>113</v>
       </c>
       <c r="B118" s="5" t="s">
-        <v>398</v>
+        <v>410</v>
       </c>
       <c r="C118" s="4" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="D118" s="9" t="s">
         <v>64</v>
       </c>
       <c r="E118" s="4" t="s">
-        <v>400</v>
+        <v>412</v>
       </c>
       <c r="F118" s="4"/>
       <c r="G118" s="4"/>
@@ -6555,7 +6651,7 @@
       <c r="L118" s="4"/>
       <c r="M118" s="7"/>
       <c r="N118" s="4" t="s">
-        <v>401</v>
+        <v>413</v>
       </c>
       <c r="O118" s="4"/>
       <c r="P118" s="4"/>
@@ -6564,43 +6660,45 @@
       <c r="S118" s="4"/>
       <c r="T118" s="7"/>
     </row>
-    <row r="119" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="119" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="4" t="n">
         <v>114</v>
       </c>
       <c r="B119" s="5" t="s">
-        <v>402</v>
+        <v>414</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="D119" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E119" s="4" t="s">
-        <v>400</v>
+        <v>412</v>
       </c>
       <c r="F119" s="4" t="s">
-        <v>399</v>
+        <v>415</v>
       </c>
       <c r="G119" s="4" t="s">
-        <v>401</v>
-      </c>
-      <c r="H119" s="7"/>
+        <v>416</v>
+      </c>
+      <c r="H119" s="7" t="s">
+        <v>417</v>
+      </c>
       <c r="I119" s="7"/>
       <c r="J119" s="4" t="s">
         <v>32</v>
       </c>
       <c r="K119" s="7"/>
       <c r="L119" s="4" t="s">
-        <v>403</v>
+        <v>418</v>
       </c>
       <c r="M119" s="7"/>
       <c r="N119" s="4" t="s">
-        <v>404</v>
+        <v>419</v>
       </c>
       <c r="O119" s="4" t="s">
-        <v>405</v>
+        <v>420</v>
       </c>
       <c r="P119" s="4" t="s">
         <v>36</v>
@@ -6621,10 +6719,10 @@
         <v>115</v>
       </c>
       <c r="B120" s="5" t="s">
-        <v>406</v>
+        <v>421</v>
       </c>
       <c r="C120" s="4" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="D120" s="6" t="s">
         <v>25</v>
@@ -6632,7 +6730,7 @@
       <c r="E120" s="4"/>
       <c r="F120" s="4"/>
       <c r="G120" s="4" t="s">
-        <v>407</v>
+        <v>422</v>
       </c>
       <c r="H120" s="7"/>
       <c r="I120" s="7"/>
@@ -6641,7 +6739,7 @@
       <c r="L120" s="4"/>
       <c r="M120" s="7"/>
       <c r="N120" s="4" t="s">
-        <v>408</v>
+        <v>423</v>
       </c>
       <c r="O120" s="4"/>
       <c r="P120" s="4"/>
@@ -6655,24 +6753,26 @@
         <v>116</v>
       </c>
       <c r="B121" s="5" t="s">
-        <v>409</v>
+        <v>424</v>
       </c>
       <c r="C121" s="4" t="s">
-        <v>410</v>
+        <v>425</v>
       </c>
       <c r="D121" s="8" t="s">
         <v>28</v>
       </c>
       <c r="E121" s="4" t="s">
+        <v>426</v>
+      </c>
+      <c r="F121" s="4" t="s">
         <v>411</v>
       </c>
-      <c r="F121" s="4" t="s">
-        <v>399</v>
-      </c>
       <c r="G121" s="4" t="s">
-        <v>372</v>
-      </c>
-      <c r="H121" s="7"/>
+        <v>383</v>
+      </c>
+      <c r="H121" s="7" t="s">
+        <v>427</v>
+      </c>
       <c r="I121" s="7"/>
       <c r="J121" s="4" t="s">
         <v>32</v>
@@ -6683,7 +6783,7 @@
       </c>
       <c r="M121" s="7"/>
       <c r="N121" s="4" t="s">
-        <v>408</v>
+        <v>423</v>
       </c>
       <c r="O121" s="4"/>
       <c r="P121" s="4" t="s">
@@ -6696,7 +6796,7 @@
         <v>124</v>
       </c>
       <c r="S121" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="T121" s="7"/>
     </row>
@@ -6705,20 +6805,20 @@
         <v>117</v>
       </c>
       <c r="B122" s="5" t="s">
-        <v>412</v>
+        <v>428</v>
       </c>
       <c r="C122" s="4" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="D122" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E122" s="4"/>
       <c r="F122" s="4" t="s">
-        <v>413</v>
+        <v>429</v>
       </c>
       <c r="G122" s="4" t="s">
-        <v>414</v>
+        <v>430</v>
       </c>
       <c r="H122" s="7"/>
       <c r="I122" s="7"/>
@@ -6739,17 +6839,17 @@
         <v>118</v>
       </c>
       <c r="B123" s="5" t="s">
-        <v>415</v>
+        <v>431</v>
       </c>
       <c r="C123" s="4" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="D123" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E123" s="4"/>
       <c r="F123" s="4" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="G123" s="4" t="s">
         <v>26</v>
@@ -6773,17 +6873,17 @@
         <v>119</v>
       </c>
       <c r="B124" s="5" t="s">
-        <v>416</v>
+        <v>432</v>
       </c>
       <c r="C124" s="4" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="D124" s="6" t="s">
         <v>25</v>
       </c>
       <c r="E124" s="4"/>
       <c r="F124" s="4" t="s">
-        <v>417</v>
+        <v>433</v>
       </c>
       <c r="G124" s="4" t="s">
         <v>44</v>
@@ -6807,10 +6907,10 @@
         <v>120</v>
       </c>
       <c r="B125" s="5" t="s">
-        <v>418</v>
+        <v>434</v>
       </c>
       <c r="C125" s="4" t="s">
-        <v>419</v>
+        <v>435</v>
       </c>
       <c r="D125" s="6" t="s">
         <v>25</v>
@@ -6818,7 +6918,7 @@
       <c r="E125" s="4"/>
       <c r="F125" s="4"/>
       <c r="G125" s="4" t="s">
-        <v>420</v>
+        <v>436</v>
       </c>
       <c r="H125" s="7"/>
       <c r="I125" s="7"/>
@@ -6839,10 +6939,10 @@
         <v>121</v>
       </c>
       <c r="B126" s="5" t="s">
-        <v>421</v>
+        <v>437</v>
       </c>
       <c r="C126" s="4" t="s">
-        <v>419</v>
+        <v>435</v>
       </c>
       <c r="D126" s="6" t="s">
         <v>25</v>
@@ -6850,7 +6950,7 @@
       <c r="E126" s="4"/>
       <c r="F126" s="4"/>
       <c r="G126" s="4" t="s">
-        <v>422</v>
+        <v>438</v>
       </c>
       <c r="H126" s="7"/>
       <c r="I126" s="7"/>
@@ -6871,10 +6971,10 @@
         <v>122</v>
       </c>
       <c r="B127" s="5" t="s">
-        <v>423</v>
+        <v>439</v>
       </c>
       <c r="C127" s="4" t="s">
-        <v>419</v>
+        <v>435</v>
       </c>
       <c r="D127" s="6" t="s">
         <v>25</v>
@@ -6882,7 +6982,7 @@
       <c r="E127" s="4"/>
       <c r="F127" s="4"/>
       <c r="G127" s="4" t="s">
-        <v>424</v>
+        <v>440</v>
       </c>
       <c r="H127" s="7"/>
       <c r="I127" s="7"/>
@@ -6903,20 +7003,20 @@
         <v>123</v>
       </c>
       <c r="B128" s="5" t="s">
-        <v>425</v>
+        <v>441</v>
       </c>
       <c r="C128" s="4" t="s">
-        <v>419</v>
+        <v>435</v>
       </c>
       <c r="D128" s="9" t="s">
         <v>64</v>
       </c>
       <c r="E128" s="4" t="s">
-        <v>426</v>
+        <v>442</v>
       </c>
       <c r="F128" s="4"/>
       <c r="G128" s="4" t="s">
-        <v>427</v>
+        <v>443</v>
       </c>
       <c r="H128" s="7"/>
       <c r="I128" s="7"/>
@@ -6937,7 +7037,7 @@
         <v>124</v>
       </c>
       <c r="B129" s="5" t="s">
-        <v>428</v>
+        <v>444</v>
       </c>
       <c r="C129" s="4" t="s">
         <v>160</v>
@@ -6971,7 +7071,7 @@
         <v>125</v>
       </c>
       <c r="B130" s="5" t="s">
-        <v>429</v>
+        <v>445</v>
       </c>
       <c r="C130" s="4" t="s">
         <v>160</v>
@@ -7005,7 +7105,7 @@
         <v>126</v>
       </c>
       <c r="B131" s="5" t="s">
-        <v>430</v>
+        <v>446</v>
       </c>
       <c r="C131" s="4" t="s">
         <v>160</v>
@@ -7014,15 +7114,17 @@
         <v>76</v>
       </c>
       <c r="E131" s="4" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="F131" s="4" t="s">
         <v>160</v>
       </c>
       <c r="G131" s="4" t="s">
-        <v>431</v>
-      </c>
-      <c r="H131" s="7"/>
+        <v>447</v>
+      </c>
+      <c r="H131" s="7" t="s">
+        <v>315</v>
+      </c>
       <c r="I131" s="7"/>
       <c r="J131" s="4" t="s">
         <v>32</v>
@@ -7033,20 +7135,20 @@
       </c>
       <c r="M131" s="7"/>
       <c r="N131" s="4" t="s">
-        <v>432</v>
+        <v>448</v>
       </c>
       <c r="O131" s="4"/>
       <c r="P131" s="4" t="s">
         <v>36</v>
       </c>
       <c r="Q131" s="4" t="s">
-        <v>433</v>
+        <v>449</v>
       </c>
       <c r="R131" s="4" t="s">
-        <v>434</v>
+        <v>450</v>
       </c>
       <c r="S131" s="4" t="s">
-        <v>435</v>
+        <v>451</v>
       </c>
       <c r="T131" s="7"/>
     </row>
@@ -7055,7 +7157,7 @@
         <v>127</v>
       </c>
       <c r="B132" s="5" t="s">
-        <v>436</v>
+        <v>452</v>
       </c>
       <c r="C132" s="4" t="s">
         <v>160</v>
@@ -7089,7 +7191,7 @@
         <v>128</v>
       </c>
       <c r="B133" s="5" t="s">
-        <v>437</v>
+        <v>453</v>
       </c>
       <c r="C133" s="4" t="s">
         <v>160</v>
@@ -7120,7 +7222,7 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B135" s="11" t="s">
-        <v>438</v>
+        <v>454</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7161,16 +7263,16 @@
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B140" s="12" t="s">
-        <v>439</v>
+        <v>455</v>
       </c>
       <c r="C140" s="12" t="str">
         <f aca="false">COUNTA($H$6:$H$133)&amp;" / "&amp;ROWS($H$6:$H$133)</f>
-        <v>12 / 128</v>
+        <v>28 / 128</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B141" s="12" t="s">
-        <v>440</v>
+        <v>456</v>
       </c>
       <c r="C141" s="12" t="n">
         <f aca="false">COUNTIFS($D$6:$D$133,"KEEP",$L$6:$L$133,"?*")</f>
@@ -7179,21 +7281,21 @@
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B143" s="11" t="s">
-        <v>441</v>
+        <v>457</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B144" s="13" t="s">
-        <v>442</v>
+        <v>458</v>
       </c>
       <c r="C144" s="13" t="s">
-        <v>443</v>
+        <v>459</v>
       </c>
       <c r="D144" s="13" t="s">
-        <v>444</v>
+        <v>460</v>
       </c>
       <c r="E144" s="13" t="s">
-        <v>445</v>
+        <v>461</v>
       </c>
       <c r="H144" s="13" t="s">
         <v>10</v>
@@ -7201,93 +7303,123 @@
     </row>
     <row r="145" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B145" s="14" t="s">
-        <v>169</v>
+        <v>317</v>
       </c>
       <c r="C145" s="14" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D145" s="14" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="E145" s="14" t="s">
-        <v>446</v>
+        <v>462</v>
       </c>
       <c r="H145" s="15"/>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B146" s="14" t="s">
-        <v>447</v>
+        <v>463</v>
       </c>
       <c r="C146" s="14" t="s">
-        <v>448</v>
+        <v>464</v>
       </c>
       <c r="D146" s="14" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="E146" s="14" t="s">
-        <v>449</v>
+        <v>465</v>
       </c>
       <c r="H146" s="15"/>
     </row>
-    <row r="147" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="147" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B147" s="14" t="s">
-        <v>450</v>
+        <v>466</v>
       </c>
       <c r="C147" s="14" t="s">
-        <v>136</v>
+        <v>415</v>
       </c>
       <c r="D147" s="14" t="s">
-        <v>448</v>
+        <v>275</v>
       </c>
       <c r="E147" s="14" t="s">
-        <v>451</v>
+        <v>467</v>
       </c>
       <c r="H147" s="15"/>
     </row>
-    <row r="148" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="148" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B148" s="14" t="s">
-        <v>452</v>
+        <v>468</v>
       </c>
       <c r="C148" s="14" t="s">
-        <v>131</v>
+        <v>359</v>
       </c>
       <c r="D148" s="14" t="s">
-        <v>210</v>
+        <v>160</v>
       </c>
       <c r="E148" s="14" t="s">
-        <v>453</v>
+        <v>469</v>
       </c>
       <c r="H148" s="15"/>
     </row>
     <row r="149" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B149" s="14" t="s">
-        <v>323</v>
+        <v>470</v>
       </c>
       <c r="C149" s="14" t="s">
-        <v>454</v>
+        <v>136</v>
       </c>
       <c r="D149" s="14" t="s">
-        <v>271</v>
+        <v>464</v>
       </c>
       <c r="E149" s="14" t="s">
-        <v>455</v>
+        <v>471</v>
       </c>
       <c r="H149" s="15"/>
     </row>
-    <row r="150" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="150" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B150" s="14" t="s">
-        <v>456</v>
+        <v>472</v>
       </c>
       <c r="C150" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="D150" s="14" t="s">
+        <v>211</v>
+      </c>
+      <c r="E150" s="14" t="s">
+        <v>473</v>
+      </c>
+      <c r="H150" s="15"/>
+    </row>
+    <row r="151" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B151" s="14" t="s">
+        <v>329</v>
+      </c>
+      <c r="C151" s="14" t="s">
+        <v>474</v>
+      </c>
+      <c r="D151" s="14" t="s">
+        <v>275</v>
+      </c>
+      <c r="E151" s="14" t="s">
+        <v>475</v>
+      </c>
+      <c r="H151" s="15"/>
+    </row>
+    <row r="152" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B152" s="14" t="s">
+        <v>476</v>
+      </c>
+      <c r="C152" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="D150" s="14" t="s">
-        <v>457</v>
-      </c>
-      <c r="E150" s="14" t="s">
-        <v>458</v>
-      </c>
-      <c r="H150" s="15"/>
+      <c r="D152" s="14" t="s">
+        <v>477</v>
+      </c>
+      <c r="E152" s="14" t="s">
+        <v>478</v>
+      </c>
+      <c r="H152" s="15"/>
     </row>
   </sheetData>
   <autoFilter ref="A5:T133"/>
@@ -7334,12 +7466,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>459</v>
+        <v>479</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>460</v>
+        <v>480</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -7349,16 +7481,16 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>461</v>
+        <v>481</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>462</v>
+        <v>482</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>463</v>
+        <v>483</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>464</v>
+        <v>484</v>
       </c>
       <c r="E4" s="13" t="s">
         <v>10</v>
@@ -7369,13 +7501,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>465</v>
+        <v>485</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>35</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="7"/>
@@ -7383,61 +7515,61 @@
     </row>
     <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>465</v>
+        <v>485</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>466</v>
+        <v>486</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>124</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>467</v>
+        <v>487</v>
       </c>
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
     </row>
     <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>465</v>
+        <v>485</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>468</v>
+        <v>488</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>124</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>467</v>
+        <v>487</v>
       </c>
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
     </row>
     <row r="8" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>465</v>
+        <v>485</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>469</v>
+        <v>489</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>124</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>467</v>
+        <v>487</v>
       </c>
       <c r="E8" s="7"/>
       <c r="F8" s="7"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>470</v>
+        <v>490</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>35</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="D9" s="4"/>
       <c r="E9" s="7"/>
@@ -7445,7 +7577,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>470</v>
+        <v>490</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>159</v>
@@ -7459,13 +7591,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>470</v>
+        <v>490</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="D11" s="4"/>
       <c r="E11" s="7"/>
@@ -7473,13 +7605,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>471</v>
+        <v>491</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>35</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="D12" s="4"/>
       <c r="E12" s="7"/>
@@ -7487,93 +7619,93 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>471</v>
+        <v>491</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>472</v>
+        <v>492</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>473</v>
+        <v>493</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>474</v>
+        <v>494</v>
       </c>
       <c r="E13" s="7"/>
       <c r="F13" s="7"/>
     </row>
     <row r="14" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>471</v>
+        <v>491</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>475</v>
+        <v>495</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>124</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>467</v>
+        <v>487</v>
       </c>
       <c r="E14" s="7"/>
       <c r="F14" s="7"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>476</v>
+        <v>496</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>472</v>
+        <v>492</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>473</v>
+        <v>493</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>474</v>
+        <v>494</v>
       </c>
       <c r="E15" s="7"/>
       <c r="F15" s="7"/>
     </row>
     <row r="16" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>476</v>
+        <v>496</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>477</v>
+        <v>468</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>124</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>467</v>
+        <v>487</v>
       </c>
       <c r="E16" s="7"/>
       <c r="F16" s="7"/>
     </row>
     <row r="17" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>476</v>
+        <v>496</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>478</v>
+        <v>497</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>124</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>467</v>
+        <v>487</v>
       </c>
       <c r="E17" s="7"/>
       <c r="F17" s="7"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>479</v>
+        <v>498</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>35</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="D18" s="4"/>
       <c r="E18" s="7"/>
@@ -7581,29 +7713,29 @@
     </row>
     <row r="19" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>479</v>
+        <v>498</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>468</v>
+        <v>488</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>124</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>467</v>
+        <v>487</v>
       </c>
       <c r="E19" s="7"/>
       <c r="F19" s="7"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>479</v>
+        <v>498</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="7"/>
@@ -7611,13 +7743,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>479</v>
+        <v>498</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>480</v>
+        <v>499</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>369</v>
+        <v>380</v>
       </c>
       <c r="D21" s="4"/>
       <c r="E21" s="7"/>
@@ -7625,80 +7757,80 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>481</v>
+        <v>500</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>472</v>
+        <v>492</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>473</v>
+        <v>493</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>474</v>
+        <v>494</v>
       </c>
       <c r="E22" s="7"/>
       <c r="F22" s="7"/>
     </row>
     <row r="23" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>481</v>
+        <v>500</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>468</v>
+        <v>488</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>124</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>467</v>
+        <v>487</v>
       </c>
       <c r="E23" s="7"/>
       <c r="F23" s="7"/>
     </row>
     <row r="24" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>481</v>
+        <v>500</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>482</v>
+        <v>501</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>124</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>467</v>
+        <v>487</v>
       </c>
       <c r="E24" s="7"/>
       <c r="F24" s="7"/>
     </row>
     <row r="25" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>481</v>
+        <v>500</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>483</v>
+        <v>502</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>124</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>467</v>
+        <v>487</v>
       </c>
       <c r="E25" s="7"/>
       <c r="F25" s="7"/>
     </row>
     <row r="26" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>481</v>
+        <v>500</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>475</v>
+        <v>495</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>124</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>467</v>
+        <v>487</v>
       </c>
       <c r="E26" s="7"/>
       <c r="F26" s="7"/>
@@ -7722,7 +7854,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -7733,185 +7865,199 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>484</v>
+        <v>503</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>485</v>
+        <v>504</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>487</v>
+        <v>506</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>488</v>
+        <v>507</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>489</v>
+        <v>508</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>490</v>
+        <v>509</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>491</v>
+        <v>510</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>492</v>
+        <v>511</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>493</v>
+        <v>512</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>494</v>
+        <v>513</v>
       </c>
       <c r="D3" s="7"/>
     </row>
     <row r="4" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>495</v>
+        <v>514</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>496</v>
+        <v>515</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>497</v>
+        <v>516</v>
       </c>
       <c r="D4" s="7"/>
     </row>
     <row r="5" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>498</v>
+        <v>517</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>499</v>
+        <v>518</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>500</v>
+        <v>519</v>
       </c>
       <c r="D5" s="7"/>
     </row>
     <row r="6" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>501</v>
+        <v>520</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>503</v>
+        <v>522</v>
       </c>
       <c r="D6" s="7"/>
     </row>
     <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>504</v>
+        <v>523</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>505</v>
+        <v>524</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>506</v>
+        <v>525</v>
       </c>
       <c r="D7" s="7"/>
     </row>
     <row r="8" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>507</v>
+        <v>526</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>508</v>
+        <v>527</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>509</v>
+        <v>528</v>
       </c>
       <c r="D8" s="7"/>
     </row>
     <row r="9" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>510</v>
+        <v>529</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>511</v>
+        <v>530</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>512</v>
+        <v>531</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>513</v>
+        <v>532</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>514</v>
+        <v>533</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>515</v>
+        <v>534</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>516</v>
+        <v>535</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>517</v>
+        <v>536</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>518</v>
+        <v>537</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>519</v>
+        <v>538</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>520</v>
+        <v>539</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>521</v>
+        <v>540</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>522</v>
+        <v>541</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>523</v>
+        <v>542</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>524</v>
+        <v>543</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>525</v>
+        <v>544</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>526</v>
+        <v>545</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>527</v>
+        <v>546</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>528</v>
+        <v>547</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>530</v>
+        <v>549</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>531</v>
+        <v>550</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>532</v>
-      </c>
-      <c r="D14" s="7"/>
+        <v>551</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>553</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>554</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>555</v>
+      </c>
+      <c r="D15" s="7"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>